<commit_message>
requirements + report update
</commit_message>
<xml_diff>
--- a/src/my_studysmart.xlsx
+++ b/src/my_studysmart.xlsx
@@ -7,7 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="exams" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="commitments" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -16,7 +17,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
+  </numFmts>
   <fonts count="2">
     <font>
       <name val="Calibri"/>
@@ -55,11 +59,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -458,13 +463,61 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D2" t="inlineStr"/>
+        <v>23</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Chapter 1, Chapter 2</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>hours</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>46169</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>lecture</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>4</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
fixed style mistakes, removed unnecessary legend code and fixed load_exam in app.py
</commit_message>
<xml_diff>
--- a/src/my_studysmart.xlsx
+++ b/src/my_studysmart.xlsx
@@ -453,16 +453,16 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Statistics</t>
+          <t>Neuroimaging</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>20</v>
+        <v>45</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -478,33 +478,37 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Action Potentials, Neuroanatomy, Sensory Systems</t>
+          <t>Action Potentials, Neuroanatomy, Sensory systems</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Biology</t>
+          <t>Statistics</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>25</v>
-      </c>
-      <c r="D4" t="inlineStr"/>
+        <v>50</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7, 8</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>